<commit_message>
🪙 BTC Momentum Score v3.0 — 13/09/2026 05:02 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 12/09/2026 04:48 UTC  |  BD1: 2026-09-05  |  BD2: 2026-09-10</t>
+          <t>Run: 13/09/2026 05:02 UTC  |  BD1: 2026-09-06  |  BD2: 2026-09-11</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>68.97</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.23999999999999</v>
+        <v>69.92</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>3.3</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>76568.10000000001</v>
+        <v>77173.8</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>92.3</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>77.59999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>77.59999999999999</v>
+        <v>74.2</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
@@ -659,10 +659,10 @@
         <v>85</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 14/09/2026 05:11 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 13/09/2026 05:02 UTC  |  BD1: 2026-09-06  |  BD2: 2026-09-11</t>
+          <t>Run: 14/09/2026 05:11 UTC  |  BD1: 2026-09-07  |  BD2: 2026-09-12</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>67.65000000000001</v>
+        <v>70.08</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>69.92</v>
+        <v>72.36</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-0.08</v>
+        <v>6.74</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>77173.8</v>
+        <v>77270.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>94.40000000000001</v>
+        <v>91</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>74.2</v>
+        <v>75.8</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>74.2</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>14</v>
+        <v>11.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.4</v>
+        <v>10</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -659,10 +659,10 @@
         <v>85</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>50</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 15/09/2026 05:05 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 14/09/2026 05:11 UTC  |  BD1: 2026-09-07  |  BD2: 2026-09-12</t>
+          <t>Run: 15/09/2026 05:05 UTC  |  BD1: 2026-09-08  |  BD2: 2026-09-13</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>70.08</v>
+        <v>69.39</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72.36</v>
+        <v>69.39</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>6.74</v>
+        <v>-5.23</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>77270.5</v>
+        <v>76838.2</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>91</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>75.8</v>
+        <v>73.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>75.8</v>
+        <v>73.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.5</v>
+        <v>12.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>100</v>
@@ -659,10 +659,10 @@
         <v>85</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 16/09/2026 05:00 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 15/09/2026 05:05 UTC  |  BD1: 2026-09-08  |  BD2: 2026-09-13</t>
+          <t>Run: 16/09/2026 05:00 UTC  |  BD1: 2026-09-09  |  BD2: 2026-09-14</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>69.39</v>
+        <v>71.17</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>69.39</v>
+        <v>71.17</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-5.23</v>
+        <v>-7.72</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>76838.2</v>
+        <v>78163.39999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>84.59999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>73.3</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>73.3</v>
+        <v>77.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>12.4</v>
+        <v>10.6</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="12">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 17/09/2026 05:03 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 16/09/2026 05:00 UTC  |  BD1: 2026-09-09  |  BD2: 2026-09-14</t>
+          <t>Run: 17/09/2026 05:03 UTC  |  BD1: 2026-09-10  |  BD2: 2026-09-15</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>71.17</v>
+        <v>66.39</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.17</v>
+        <v>66.39</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-7.72</v>
+        <v>-8.449999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>78163.39999999999</v>
+        <v>75612.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>84.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>77.59999999999999</v>
+        <v>70.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>77.59999999999999</v>
+        <v>70.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>10.6</v>
+        <v>11.1</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>6.3</v>
+        <v>7.7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>6.3</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>
@@ -659,10 +659,10 @@
         <v>85</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 18/09/2026 04:56 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 17/09/2026 05:03 UTC  |  BD1: 2026-09-10  |  BD2: 2026-09-15</t>
+          <t>Run: 18/09/2026 04:56 UTC  |  BD1: 2026-09-11  |  BD2: 2026-09-16</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>66.39</v>
+        <v>65.05</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>66.39</v>
+        <v>65.05</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-8.449999999999999</v>
+        <v>-5.11</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>75612.5</v>
+        <v>76150.3</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>77.59999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>70.3</v>
+        <v>72.5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>70.3</v>
+        <v>72.5</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 19/09/2026 04:47 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 18/09/2026 04:56 UTC  |  BD1: 2026-09-11  |  BD2: 2026-09-16</t>
+          <t>Run: 19/09/2026 04:47 UTC  |  BD1: 2026-09-12  |  BD2: 2026-09-17</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>65.05</v>
+        <v>63.74</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>65.05</v>
+        <v>63.74</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-5.11</v>
+        <v>-19.43</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>76150.3</v>
+        <v>76403.8</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>74.2</v>
+        <v>75.8</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>72.5</v>
+        <v>72.2</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>72.5</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.4</v>
+        <v>10</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 20/09/2026 05:05 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 19/09/2026 04:47 UTC  |  BD1: 2026-09-12  |  BD2: 2026-09-17</t>
+          <t>Run: 20/09/2026 05:05 UTC  |  BD1: 2026-09-13  |  BD2: 2026-09-18</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>63.74</v>
+        <v>74.31</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>63.74</v>
+        <v>74.31</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-19.43</v>
+        <v>15.07</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>76403.8</v>
+        <v>80901.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>75.8</v>
+        <v>73.3</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>72.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>72.2</v>
+        <v>90.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>10</v>
+        <v>7.3</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>7</v>
+        <v>10.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>7</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -656,13 +656,13 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 21/09/2026 05:10 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 20/09/2026 05:05 UTC  |  BD1: 2026-09-13  |  BD2: 2026-09-18</t>
+          <t>Run: 21/09/2026 05:10 UTC  |  BD1: 2026-09-14  |  BD2: 2026-09-19</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>74.31</v>
+        <v>74.52</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74.31</v>
+        <v>74.52</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>15.07</v>
+        <v>14.43</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>80901.5</v>
+        <v>81233.7</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>73.3</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>90.59999999999999</v>
+        <v>90</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>90.59999999999999</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 22/09/2026 05:11 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 21/09/2026 05:10 UTC  |  BD1: 2026-09-14  |  BD2: 2026-09-19</t>
+          <t>Run: 22/09/2026 05:11 UTC  |  BD1: 2026-09-15  |  BD2: 2026-09-20</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>74.52</v>
+        <v>71.94</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74.52</v>
+        <v>71.94</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>14.43</v>
+        <v>19.56</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81233.7</v>
+        <v>81142.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>77.59999999999999</v>
+        <v>70.3</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>90</v>
+        <v>91.2</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>90</v>
+        <v>91.2</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>6.3</v>
+        <v>7.7</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>10.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>10.4</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 23/09/2026 04:56 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 22/09/2026 05:11 UTC  |  BD1: 2026-09-15  |  BD2: 2026-09-20</t>
+          <t>Run: 23/09/2026 04:56 UTC  |  BD1: 2026-09-16  |  BD2: 2026-09-21</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>71.94</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.94</v>
+        <v>71.31999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>19.56</v>
+        <v>17.65</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81142.60000000001</v>
+        <v>86602.89999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>70.3</v>
+        <v>72.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>91.2</v>
+        <v>97.5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>91.2</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>9.199999999999999</v>
+        <v>13.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>9.199999999999999</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="12">
@@ -643,10 +643,10 @@
         <v>90</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 24/09/2026 05:06 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 23/09/2026 04:56 UTC  |  BD1: 2026-09-16  |  BD2: 2026-09-21</t>
+          <t>Run: 24/09/2026 05:06 UTC  |  BD1: 2026-09-17  |  BD2: 2026-09-22</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>71.31999999999999</v>
+        <v>64.63</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.31999999999999</v>
+        <v>64.63</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>17.65</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>86602.89999999999</v>
+        <v>86172.3</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>72.5</v>
+        <v>72.2</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>97.5</v>
+        <v>95.7</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>97.5</v>
+        <v>95.7</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>13.4</v>
+        <v>15.7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>13.4</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 25/09/2026 05:08 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 24/09/2026 05:06 UTC  |  BD1: 2026-09-17  |  BD2: 2026-09-22</t>
+          <t>Run: 25/09/2026 05:08 UTC  |  BD1: 2026-09-18  |  BD2: 2026-09-23</t>
         </is>
       </c>
     </row>
@@ -509,11 +509,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>64.63</v>
+        <v>80.84</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Moderate ↑</t>
+          <t>Strong ↑</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64.63</v>
+        <v>80.84</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>21.2</v>
+        <v>-2.02</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>86172.3</v>
+        <v>84383</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>72.2</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>95.7</v>
+        <v>91.7</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>95.7</v>
+        <v>91.7</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>7</v>
+        <v>10.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>15.7</v>
+        <v>17.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>15.7</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 26/09/2026 05:12 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 25/09/2026 05:08 UTC  |  BD1: 2026-09-18  |  BD2: 2026-09-23</t>
+          <t>Run: 26/09/2026 05:12 UTC  |  BD1: 2026-09-19  |  BD2: 2026-09-24</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>80.84</v>
+        <v>79.84999999999999</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80.84</v>
+        <v>79.84999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-2.02</v>
+        <v>-3.75</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84383</v>
+        <v>84379.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>90.59999999999999</v>
+        <v>90</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>91.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>91.7</v>
+        <v>89.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>10.5</v>
+        <v>10.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>17.3</v>
+        <v>18.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>17.3</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
@@ -643,10 +643,10 @@
         <v>90</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 27/09/2026 05:29 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 26/09/2026 05:12 UTC  |  BD1: 2026-09-19  |  BD2: 2026-09-24</t>
+          <t>Run: 27/09/2026 05:29 UTC  |  BD1: 2026-09-20  |  BD2: 2026-09-25</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>79.84999999999999</v>
+        <v>82.48</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.84999999999999</v>
+        <v>82.48</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-3.75</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84379.10000000001</v>
+        <v>84034.89999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>90</v>
+        <v>91.2</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>89.59999999999999</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>89.59999999999999</v>
+        <v>90.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>10.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 28/09/2026 05:38 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 27/09/2026 05:29 UTC  |  BD1: 2026-09-20  |  BD2: 2026-09-25</t>
+          <t>Run: 28/09/2026 05:38 UTC  |  BD1: 2026-09-21  |  BD2: 2026-09-26</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>82.48</v>
+        <v>81.08</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>82.48</v>
+        <v>81.08</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.53</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84034.89999999999</v>
+        <v>84406.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>91.2</v>
+        <v>97.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>90.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>90.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>9.199999999999999</v>
+        <v>13.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>19.1</v>
+        <v>16.2</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>19.1</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="12">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 29/09/2026 05:55 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 28/09/2026 05:38 UTC  |  BD1: 2026-09-21  |  BD2: 2026-09-26</t>
+          <t>Run: 29/09/2026 05:55 UTC  |  BD1: 2026-09-22  |  BD2: 2026-09-27</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>81.08</v>
+        <v>76.01000000000001</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>81.08</v>
+        <v>76.01000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.87</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84406.5</v>
+        <v>84458.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>97.5</v>
+        <v>95.7</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>85.90000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>85.90000000000001</v>
+        <v>86.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>13.4</v>
+        <v>15.7</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 30/09/2026 05:45 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 29/09/2026 05:55 UTC  |  BD1: 2026-09-22  |  BD2: 2026-09-27</t>
+          <t>Run: 30/09/2026 05:45 UTC  |  BD1: 2026-09-23  |  BD2: 2026-09-28</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>76.01000000000001</v>
+        <v>81.13</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>76.01000000000001</v>
+        <v>81.13</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.57</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84458.10000000001</v>
+        <v>83502.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>95.7</v>
+        <v>91.7</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>86.40000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>86.40000000000001</v>
+        <v>88.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>15.7</v>
+        <v>17.3</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>14.4</v>
+        <v>16.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>14.4</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 01/10/2026 06:19 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 30/09/2026 05:45 UTC  |  BD1: 2026-09-23  |  BD2: 2026-09-28</t>
+          <t>Run: 01/10/2026 06:19 UTC  |  BD1: 2026-09-24  |  BD2: 2026-09-29</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>81.13</v>
+        <v>77.75</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>81.13</v>
+        <v>77.75</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>2.59</v>
+        <v>-0.46</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>83502.60000000001</v>
+        <v>83622.39999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>91.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>88.09999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>88.09999999999999</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>17.3</v>
+        <v>18.3</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>16.5</v>
+        <v>14.8</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>16.5</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>90</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 02/10/2026 05:56 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 01/10/2026 06:19 UTC  |  BD1: 2026-09-24  |  BD2: 2026-09-29</t>
+          <t>Run: 02/10/2026 05:56 UTC  |  BD1: 2026-09-25  |  BD2: 2026-09-30</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>77.75</v>
+        <v>80.48</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>77.75</v>
+        <v>80.48</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-0.46</v>
+        <v>-5.52</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>83622.39999999999</v>
+        <v>83553.89999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>89.59999999999999</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>90.3</v>
+        <v>90.5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>90.3</v>
+        <v>90.5</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>14.8</v>
+        <v>15.8</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>14.8</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>70</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 03/10/2026 05:30 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 02/10/2026 05:56 UTC  |  BD1: 2026-09-25  |  BD2: 2026-09-30</t>
+          <t>Run: 03/10/2026 05:30 UTC  |  BD1: 2026-09-26  |  BD2: 2026-10-01</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>80.48</v>
+        <v>80.22</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80.48</v>
+        <v>80.22</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-5.52</v>
+        <v>-3.59</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>83553.89999999999</v>
+        <v>84853.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>90.40000000000001</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>90.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>90.5</v>
+        <v>93.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>19.1</v>
+        <v>16.2</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>15.8</v>
+        <v>17.2</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>15.8</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 04/10/2026 06:05 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 03/10/2026 05:30 UTC  |  BD1: 2026-09-26  |  BD2: 2026-10-01</t>
+          <t>Run: 04/10/2026 06:05 UTC  |  BD1: 2026-09-27  |  BD2: 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>80.22</v>
+        <v>80.37</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80.22</v>
+        <v>80.37</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-3.59</v>
+        <v>7.15</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84853.10000000001</v>
+        <v>84497.2</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>85.90000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>93.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>93.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>16.2</v>
+        <v>14.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>17.2</v>
+        <v>20.8</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>17.2</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="C12" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="C12" s="9" t="n">
-        <v>70</v>
-      </c>
       <c r="D12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 05/10/2026 05:59 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 04/10/2026 06:05 UTC  |  BD1: 2026-09-27  |  BD2: 2026-10-02</t>
+          <t>Run: 05/10/2026 05:59 UTC  |  BD1: 2026-09-28  |  BD2: 2026-10-03</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>80.37</v>
+        <v>83.09</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80.37</v>
+        <v>83.09</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7.15</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84497.2</v>
+        <v>84763.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>86.40000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>92.90000000000001</v>
+        <v>94.5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>92.90000000000001</v>
+        <v>94.5</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>14.4</v>
+        <v>16.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>20.8</v>
+        <v>18</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>20.8</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 06/10/2026 06:36 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 05/10/2026 05:59 UTC  |  BD1: 2026-09-28  |  BD2: 2026-10-03</t>
+          <t>Run: 06/10/2026 06:36 UTC  |  BD1: 2026-09-29  |  BD2: 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>83.09</v>
+        <v>78.19</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>83.09</v>
+        <v>78.19</v>
       </c>
     </row>
     <row r="6">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84763.60000000001</v>
+        <v>86480.3</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>88.09999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>94.5</v>
+        <v>96.5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>94.5</v>
+        <v>96.5</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>16.5</v>
+        <v>14.8</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>18</v>
+        <v>16.7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>18</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 07/10/2026 06:14 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 06/10/2026 06:36 UTC  |  BD1: 2026-09-29  |  BD2: 2026-10-04</t>
+          <t>Run: 07/10/2026 06:14 UTC  |  BD1: 2026-09-30  |  BD2: 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>78.19</v>
+        <v>78.92</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>78.19</v>
+        <v>78.92</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.34</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>86480.3</v>
+        <v>85786.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>90.3</v>
+        <v>90.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>96.5</v>
+        <v>95.2</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>96.5</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>14.8</v>
+        <v>15.8</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>16.7</v>
+        <v>15.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>16.7</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>70</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 08/10/2026 06:22 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 07/10/2026 06:14 UTC  |  BD1: 2026-09-30  |  BD2: 2026-10-05</t>
+          <t>Run: 08/10/2026 06:22 UTC  |  BD1: 2026-10-01  |  BD2: 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>78.92</v>
+        <v>78.98</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>78.92</v>
+        <v>78.98</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>2.39</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>85786.60000000001</v>
+        <v>85557.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>90.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>95.2</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>95.2</v>
+        <v>93.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>15.8</v>
+        <v>17.2</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>15.5</v>
+        <v>13.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>15.5</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 09/10/2026 06:24 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 08/10/2026 06:22 UTC  |  BD1: 2026-10-01  |  BD2: 2026-10-06</t>
+          <t>Run: 09/10/2026 06:24 UTC  |  BD1: 2026-10-02  |  BD2: 2026-10-07</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>78.98</v>
+        <v>81.23999999999999</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>78.98</v>
+        <v>81.23999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.12</v>
+        <v>-5.41</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>85557.60000000001</v>
+        <v>83275.89999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>93.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>93.90000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>93.90000000000001</v>
+        <v>87.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>17.2</v>
+        <v>20.8</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 10/10/2026 06:05 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 09/10/2026 06:24 UTC  |  BD1: 2026-10-02  |  BD2: 2026-10-07</t>
+          <t>Run: 10/10/2026 06:05 UTC  |  BD1: 2026-10-03  |  BD2: 2026-10-08</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>81.23999999999999</v>
+        <v>79.67</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>81.23999999999999</v>
+        <v>79.67</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-5.41</v>
+        <v>-8.18</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>83275.89999999999</v>
+        <v>81676.3</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>92.90000000000001</v>
+        <v>94.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>87.90000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>87.90000000000001</v>
+        <v>85.7</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>20.8</v>
+        <v>18</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>13.3</v>
+        <v>17.8</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>13.3</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>100</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 11/10/2026 06:03 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 10/10/2026 06:05 UTC  |  BD1: 2026-10-03  |  BD2: 2026-10-08</t>
+          <t>Run: 11/10/2026 06:03 UTC  |  BD1: 2026-10-04  |  BD2: 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>79.67</v>
+        <v>78.65000000000001</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.67</v>
+        <v>78.65000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-8.18</v>
+        <v>-0.42</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81676.3</v>
+        <v>82546.3</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>94.5</v>
+        <v>96.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>85.7</v>
+        <v>82.5</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>85.7</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>18</v>
+        <v>16.7</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>17.8</v>
+        <v>18.2</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>17.8</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 12/10/2026 06:14 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 11/10/2026 06:03 UTC  |  BD1: 2026-10-04  |  BD2: 2026-10-09</t>
+          <t>Run: 12/10/2026 06:13 UTC  |  BD1: 2026-10-05  |  BD2: 2026-10-10</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>78.65000000000001</v>
+        <v>79.20999999999999</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>78.65000000000001</v>
+        <v>79.20999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-0.42</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>82546.3</v>
+        <v>82912.2</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>96.5</v>
+        <v>95.2</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>82.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>82.5</v>
+        <v>83.59999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>16.7</v>
+        <v>15.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>18.2</v>
+        <v>16.2</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>18.2</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 13/10/2026 06:55 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 12/10/2026 06:13 UTC  |  BD1: 2026-10-05  |  BD2: 2026-10-10</t>
+          <t>Run: 13/10/2026 06:55 UTC  |  BD1: 2026-10-06  |  BD2: 2026-10-11</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>79.20999999999999</v>
+        <v>79.70999999999999</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.20999999999999</v>
+        <v>79.70999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-1.8</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>82912.2</v>
+        <v>83679.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>95.2</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>83.59999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>83.59999999999999</v>
+        <v>84.8</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>15.5</v>
+        <v>13.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>16.2</v>
+        <v>14.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>16.2</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="12">
@@ -643,10 +643,10 @@
         <v>90</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 14/10/2026 05:07 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 13/10/2026 06:55 UTC  |  BD1: 2026-10-06  |  BD2: 2026-10-11</t>
+          <t>Run: 14/10/2026 05:07 UTC  |  BD1: 2026-10-07  |  BD2: 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -509,11 +509,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>79.70999999999999</v>
+        <v>70.03</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Strong ↑</t>
+          <t>Moderate ↑</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.70999999999999</v>
+        <v>72.31</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.34</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>83679.5</v>
+        <v>81762.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>93.90000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>84.8</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>84.8</v>
+        <v>79.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>14.5</v>
+        <v>12.4</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>14.5</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="12">
@@ -659,10 +659,10 @@
         <v>100</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 15/10/2026 04:55 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 14/10/2026 05:07 UTC  |  BD1: 2026-10-07  |  BD2: 2026-10-12</t>
+          <t>Run: 15/10/2026 04:55 UTC  |  BD1: 2026-10-08  |  BD2: 2026-10-13</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>70.03</v>
+        <v>71.29000000000001</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72.31</v>
+        <v>71.29000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-17</v>
+        <v>-8.59</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81762.60000000001</v>
+        <v>83095.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>87.90000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>79.09999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>79.09999999999999</v>
+        <v>85.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>13.3</v>
+        <v>17.8</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>12.4</v>
+        <v>11.7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>12.4</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 16/10/2026 04:45 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 15/10/2026 04:55 UTC  |  BD1: 2026-10-08  |  BD2: 2026-10-13</t>
+          <t>Run: 16/10/2026 04:45 UTC  |  BD1: 2026-10-09  |  BD2: 2026-10-14</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>71.29000000000001</v>
+        <v>70.12</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.29000000000001</v>
+        <v>72.40000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-8.59</v>
+        <v>-16.64</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>83095.10000000001</v>
+        <v>81562.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>85.7</v>
+        <v>82.5</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>85.3</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>85.3</v>
+        <v>81.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>17.8</v>
+        <v>18.2</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>80</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 17/10/2026 04:44 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 16/10/2026 04:45 UTC  |  BD1: 2026-10-09  |  BD2: 2026-10-14</t>
+          <t>Run: 17/10/2026 04:44 UTC  |  BD1: 2026-10-10  |  BD2: 2026-10-15</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>70.12</v>
+        <v>70.42</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72.40000000000001</v>
+        <v>72.69</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-16.64</v>
+        <v>-15.79</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81562.5</v>
+        <v>82141.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>82.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>81.09999999999999</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>81.09999999999999</v>
+        <v>81.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>18.2</v>
+        <v>16.2</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>12</v>
+        <v>15.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>12</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 18/10/2026 04:50 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 17/10/2026 04:44 UTC  |  BD1: 2026-10-10  |  BD2: 2026-10-15</t>
+          <t>Run: 18/10/2026 04:50 UTC  |  BD1: 2026-10-11  |  BD2: 2026-10-16</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>70.42</v>
+        <v>69.42</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>72.69</v>
+        <v>71.69</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-15.79</v>
+        <v>-20.93</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>82141.5</v>
+        <v>81500.8</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>83.59999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>81.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>81.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>16.2</v>
+        <v>14.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>15.5</v>
+        <v>16.7</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>15.5</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 19/10/2026 04:58 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 18/10/2026 04:50 UTC  |  BD1: 2026-10-11  |  BD2: 2026-10-16</t>
+          <t>Run: 19/10/2026 04:58 UTC  |  BD1: 2026-10-12  |  BD2: 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>69.42</v>
+        <v>60.22</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>71.69</v>
+        <v>64.76000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-20.93</v>
+        <v>-2.64</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81500.8</v>
+        <v>81382.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>84.8</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>79.40000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>79.40000000000001</v>
+        <v>80.7</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>14.5</v>
+        <v>12.4</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>16.7</v>
+        <v>15</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>16.7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 20/10/2026 05:03 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 19/10/2026 04:58 UTC  |  BD1: 2026-10-12  |  BD2: 2026-10-17</t>
+          <t>Run: 20/10/2026 05:03 UTC  |  BD1: 2026-10-13  |  BD2: 2026-10-18</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>60.22</v>
+        <v>62.84</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64.76000000000001</v>
+        <v>65.11</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-2.64</v>
+        <v>-8.300000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81382.10000000001</v>
+        <v>82017.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>79.09999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>80.7</v>
+        <v>80.8</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>80.7</v>
+        <v>80.8</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>12.4</v>
+        <v>11.7</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>15</v>
+        <v>13.6</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>15</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 21/10/2026 05:04 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 20/10/2026 05:03 UTC  |  BD1: 2026-10-13  |  BD2: 2026-10-18</t>
+          <t>Run: 21/10/2026 05:04 UTC  |  BD1: 2026-10-14  |  BD2: 2026-10-19</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>62.84</v>
+        <v>62.48</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>65.11</v>
+        <v>64.76000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-8.300000000000001</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>82017.60000000001</v>
+        <v>81853.5</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>85.3</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>80.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>80.8</v>
+        <v>81.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>13.6</v>
+        <v>12.1</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>13.6</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 22/10/2026 05:06 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 21/10/2026 05:04 UTC  |  BD1: 2026-10-14  |  BD2: 2026-10-19</t>
+          <t>Run: 22/10/2026 05:06 UTC  |  BD1: 2026-10-15  |  BD2: 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>62.48</v>
+        <v>64.66</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64.76000000000001</v>
+        <v>66.93000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>1.36</v>
+        <v>4.28</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81853.5</v>
+        <v>82941</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>81.09999999999999</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>81.90000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>81.90000000000001</v>
+        <v>84.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>12</v>
+        <v>15.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 23/10/2026 05:06 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 22/10/2026 05:06 UTC  |  BD1: 2026-10-15  |  BD2: 2026-10-20</t>
+          <t>Run: 23/10/2026 05:06 UTC  |  BD1: 2026-10-16  |  BD2: 2026-10-21</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>64.66</v>
+        <v>70.89</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>66.93000000000001</v>
+        <v>73.17</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4.28</v>
+        <v>23.87</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>82941</v>
+        <v>84012</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>81.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>84.3</v>
+        <v>85.7</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>84.3</v>
+        <v>85.7</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>15.5</v>
+        <v>16.7</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -659,10 +659,10 @@
         <v>25</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 24/10/2026 04:50 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 23/10/2026 05:06 UTC  |  BD1: 2026-10-16  |  BD2: 2026-10-21</t>
+          <t>Run: 24/10/2026 04:50 UTC  |  BD1: 2026-10-17  |  BD2: 2026-10-22</t>
         </is>
       </c>
     </row>
@@ -509,11 +509,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>70.89</v>
+        <v>56.98</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Moderate ↑</t>
+          <t>Neutral →</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73.17</v>
+        <v>61.53</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>23.87</v>
+        <v>-3.83</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>84012</v>
+        <v>81311.89999999999</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>79.40000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>85.7</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>85.7</v>
+        <v>75.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>16.7</v>
+        <v>15</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.3</v>
+        <v>12.6</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.3</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>60</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
@@ -627,10 +627,10 @@
         <v>100</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14">
@@ -659,10 +659,10 @@
         <v>25</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D15" s="9" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 25/10/2026 05:00 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 24/10/2026 04:50 UTC  |  BD1: 2026-10-17  |  BD2: 2026-10-22</t>
+          <t>Run: 25/10/2026 05:00 UTC  |  BD1: 2026-10-18  |  BD2: 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>56.98</v>
+        <v>56.47</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61.53</v>
+        <v>61.02</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-3.83</v>
+        <v>-4.44</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81311.89999999999</v>
+        <v>81074.2</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>80.7</v>
+        <v>80.8</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>75.09999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>75.09999999999999</v>
+        <v>71.2</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>15</v>
+        <v>13.6</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>12.6</v>
+        <v>11.6</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>12.6</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 26/10/2026 05:04 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 25/10/2026 05:00 UTC  |  BD1: 2026-10-18  |  BD2: 2026-10-23</t>
+          <t>Run: 26/10/2026 05:04 UTC  |  BD1: 2026-10-19  |  BD2: 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>56.47</v>
+        <v>58.6</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61.02</v>
+        <v>60.87</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-4.44</v>
+        <v>-9.140000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81074.2</v>
+        <v>80790.8</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>80.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>71.2</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>71.2</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>13.6</v>
+        <v>12.1</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 27/10/2026 05:19 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 26/10/2026 05:04 UTC  |  BD1: 2026-10-19  |  BD2: 2026-10-24</t>
+          <t>Run: 27/10/2026 05:19 UTC  |  BD1: 2026-10-20  |  BD2: 2026-10-25</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>58.6</v>
+        <v>58.29</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60.87</v>
+        <v>60.56</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-9.140000000000001</v>
+        <v>-17.02</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>80790.8</v>
+        <v>80024</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>81.90000000000001</v>
+        <v>84.3</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>69.90000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>69.90000000000001</v>
+        <v>66.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>12.1</v>
+        <v>11.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>11.5</v>
+        <v>9.1</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>11.5</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="C12" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="C12" s="9" t="n">
-        <v>80</v>
-      </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 28/10/2026 05:58 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 27/10/2026 05:19 UTC  |  BD1: 2026-10-20  |  BD2: 2026-10-25</t>
+          <t>Run: 28/10/2026 05:58 UTC  |  BD1: 2026-10-21  |  BD2: 2026-10-26</t>
         </is>
       </c>
     </row>
@@ -509,11 +509,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>58.29</v>
+        <v>67.81</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Neutral →</t>
+          <t>Moderate ↑</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60.56</v>
+        <v>70.08</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-17.02</v>
+        <v>-30.05</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>80024</v>
+        <v>80006.7</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>84.3</v>
+        <v>85.7</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>66.90000000000001</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>66.90000000000001</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.5</v>
+        <v>11.3</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>9.1</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="C12" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="C12" s="9" t="n">
-        <v>60</v>
-      </c>
       <c r="D12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 29/10/2026 06:05 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 28/10/2026 05:58 UTC  |  BD1: 2026-10-21  |  BD2: 2026-10-26</t>
+          <t>Run: 29/10/2026 06:05 UTC  |  BD1: 2026-10-22  |  BD2: 2026-10-27</t>
         </is>
       </c>
     </row>
@@ -509,11 +509,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>67.81</v>
+        <v>52.59</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Moderate ↑</t>
+          <t>Neutral →</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>70.08</v>
+        <v>57.14</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-30.05</v>
+        <v>-4.95</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>80006.7</v>
+        <v>80805.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>85.7</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>65.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>65.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.3</v>
+        <v>12.6</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>8.6</v>
+        <v>6.9</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>8.6</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +608,13 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>65</v>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>25</v>

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 30/10/2026 06:06 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="00FF0000"/>
+      <color rgb="0000B050"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 29/10/2026 06:05 UTC  |  BD1: 2026-10-22  |  BD2: 2026-10-27</t>
+          <t>Run: 30/10/2026 06:06 UTC  |  BD1: 2026-10-23  |  BD2: 2026-10-28</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>52.59</v>
+        <v>56.45</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57.14</v>
+        <v>58.72</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>-4.95</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>80805.10000000001</v>
+        <v>81267.60000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>75.09999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>71.09999999999999</v>
+        <v>75.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>71.09999999999999</v>
+        <v>75.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>12.6</v>
+        <v>11.6</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>6.9</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
🪙 BTC Momentum Score v3.0 — 31/10/2026 06:00 UTC
</commit_message>
<xml_diff>
--- a/BTC_Momentum_v3.0.xlsx
+++ b/BTC_Momentum_v3.0.xlsx
@@ -48,7 +48,7 @@
       <sz val="16"/>
     </font>
     <font>
-      <color rgb="0000B050"/>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <b val="1"/>
@@ -498,7 +498,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Run: 30/10/2026 06:06 UTC  |  BD1: 2026-10-23  |  BD2: 2026-10-28</t>
+          <t>Run: 31/10/2026 06:00 UTC  |  BD1: 2026-10-24  |  BD2: 2026-10-29</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>56.45</v>
+        <v>51.82</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58.72</v>
+        <v>56.36</v>
       </c>
     </row>
     <row r="6">
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4.39</v>
+        <v>-4.41</v>
       </c>
     </row>
     <row r="7">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>81267.60000000001</v>
+        <v>77775.10000000001</v>
       </c>
     </row>
     <row r="9">
@@ -576,13 +576,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>71.2</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>75.3</v>
+        <v>66.3</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>75.3</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="11">
@@ -592,13 +592,13 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>6.6</v>
+        <v>8.6</v>
       </c>
       <c r="D11" s="9" t="n">
-        <v>6.6</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="12">
@@ -611,10 +611,10 @@
         <v>80</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D12" s="9" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">

</xml_diff>